<commit_message>
minor changes to complete project
</commit_message>
<xml_diff>
--- a/outputs/clean_expenses.xlsx
+++ b/outputs/clean_expenses.xlsx
@@ -2228,7 +2228,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Rejpected</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Rejpected</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Rejpected</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Rejpected</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
@@ -11470,7 +11470,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Rejpected</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -15475,7 +15475,7 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Rejpected</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
@@ -17770,7 +17770,7 @@
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Rejpected</t>
         </is>
       </c>
       <c r="H342" t="inlineStr">
@@ -24054,7 +24054,7 @@
       </c>
       <c r="G466" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Rejpected</t>
         </is>
       </c>
       <c r="H466" t="inlineStr">

</xml_diff>